<commit_message>
Major refactor to the intended output following assement guidelines.
</commit_message>
<xml_diff>
--- a/outputs/chinese_boiler_dataset/tables/pre_forecasting_summary.xlsx
+++ b/outputs/chinese_boiler_dataset/tables/pre_forecasting_summary.xlsx
@@ -10,6 +10,9 @@
     <sheet name="granularity" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="target_distribution" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="target_transforms" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="target_autocorrelation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="target_stationarity" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="target_correlations" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -555,35 +558,6 @@
         <v>44647.60409722223</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>44652.60340277778</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>subset_B_5min</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>subset_B</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>5min</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1440</v>
-      </c>
-      <c r="E5" t="n">
-        <v>15</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>44647.606875</v>
-      </c>
-      <c r="G5" s="2" t="n">
         <v>44652.60340277778</v>
       </c>
     </row>
@@ -598,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -807,53 +781,6 @@
       </c>
       <c r="M4" t="n">
         <v>-0.2345766553598631</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>subset_B_5min</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>5min</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>TE_8313B.AV_0#</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1440</v>
-      </c>
-      <c r="E5" t="n">
-        <v>774.0630346064814</v>
-      </c>
-      <c r="F5" t="n">
-        <v>10.44418514182298</v>
-      </c>
-      <c r="G5" t="n">
-        <v>739.5895</v>
-      </c>
-      <c r="H5" t="n">
-        <v>767.8555</v>
-      </c>
-      <c r="I5" t="n">
-        <v>774.2698333333333</v>
-      </c>
-      <c r="J5" t="n">
-        <v>781.1922916666667</v>
-      </c>
-      <c r="K5" t="n">
-        <v>815.4731666666667</v>
-      </c>
-      <c r="L5" t="n">
-        <v>13.33679166666673</v>
-      </c>
-      <c r="M5" t="n">
-        <v>-0.2487446422150158</v>
       </c>
     </row>
   </sheetData>
@@ -867,7 +794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1039,34 +966,34 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>86389</v>
+        <v>86395</v>
       </c>
       <c r="E3" t="n">
-        <v>774.0631438319693</v>
+        <v>774.0631044427726</v>
       </c>
       <c r="F3" t="n">
-        <v>10.65468342157003</v>
+        <v>10.67337210764209</v>
       </c>
       <c r="G3" t="n">
-        <v>738.5091666666667</v>
+        <v>738.0649999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>767.6083333333335</v>
+        <v>767.5983333333334</v>
       </c>
       <c r="I3" t="n">
-        <v>774.3366666666667</v>
+        <v>774.3250000000002</v>
       </c>
       <c r="J3" t="n">
-        <v>781.2675</v>
+        <v>781.275</v>
       </c>
       <c r="K3" t="n">
-        <v>817.8891666666667</v>
+        <v>818.0116666666667</v>
       </c>
       <c r="L3" t="n">
-        <v>13.65916666666658</v>
+        <v>13.67666666666662</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.2347992594581003</v>
+        <v>-0.2331823403697795</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -1080,11 +1007,11 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>1min</t>
+          <t>30s</t>
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -1104,34 +1031,34 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>86341</v>
+        <v>86389</v>
       </c>
       <c r="E4" t="n">
-        <v>774.0620165989121</v>
+        <v>774.0631438319693</v>
       </c>
       <c r="F4" t="n">
-        <v>10.44573072329733</v>
+        <v>10.65468342157003</v>
       </c>
       <c r="G4" t="n">
-        <v>739.2755</v>
+        <v>738.5091666666667</v>
       </c>
       <c r="H4" t="n">
-        <v>767.7516666666667</v>
+        <v>767.6083333333335</v>
       </c>
       <c r="I4" t="n">
-        <v>774.2495</v>
+        <v>774.3366666666667</v>
       </c>
       <c r="J4" t="n">
-        <v>781.2196666666666</v>
+        <v>781.2675</v>
       </c>
       <c r="K4" t="n">
-        <v>815.6681666666666</v>
+        <v>817.8891666666667</v>
       </c>
       <c r="L4" t="n">
-        <v>13.46799999999996</v>
+        <v>13.65916666666658</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.2476865316551196</v>
+        <v>-0.2347992594581003</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -1145,11 +1072,11 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>5min</t>
+          <t>1min</t>
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -1169,34 +1096,34 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>86399</v>
+        <v>86341</v>
       </c>
       <c r="E5" t="n">
-        <v>-2.673642056042384e-05</v>
+        <v>774.0620165989121</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2732205123091537</v>
+        <v>10.44573072329733</v>
       </c>
       <c r="G5" t="n">
-        <v>-1.139999999999986</v>
+        <v>739.2755</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1700000000000728</v>
+        <v>767.7516666666667</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>774.2495</v>
       </c>
       <c r="J5" t="n">
-        <v>0.1700000000000728</v>
+        <v>781.2196666666666</v>
       </c>
       <c r="K5" t="n">
-        <v>1.299999999999955</v>
+        <v>815.6681666666666</v>
       </c>
       <c r="L5" t="n">
-        <v>0.3400000000001455</v>
+        <v>13.46799999999996</v>
       </c>
       <c r="M5" t="n">
-        <v>0.03859649943443079</v>
+        <v>-0.2476865316551196</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -1205,16 +1132,16 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>first_difference</t>
+          <t>trailing_rolling_mean</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>5min</t>
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -1234,34 +1161,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>86398</v>
+        <v>86399</v>
       </c>
       <c r="E6" t="n">
-        <v>2.777842079677876e-06</v>
+        <v>-2.673642056042384e-05</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1383208577587473</v>
+        <v>0.2732205123091537</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.57000000000005</v>
+        <v>-1.139999999999986</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.09999999999990905</v>
+        <v>-0.1700000000000728</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0.09999999999990905</v>
+        <v>0.1700000000000728</v>
       </c>
       <c r="K6" t="n">
-        <v>0.7000000000000455</v>
+        <v>1.299999999999955</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1999999999998181</v>
+        <v>0.3400000000001455</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0734800260731755</v>
+        <v>0.03859649943443079</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -1270,7 +1197,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>second_difference</t>
+          <t>first_difference</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1285,12 +1212,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>subset_B_30s</t>
+          <t>subset_B_raw</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>30s</t>
+          <t>raw</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1299,34 +1226,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>14400</v>
+        <v>86398</v>
       </c>
       <c r="E7" t="n">
-        <v>774.0630346064816</v>
+        <v>2.777842079677876e-06</v>
       </c>
       <c r="F7" t="n">
-        <v>10.67342310535531</v>
+        <v>0.1383208577587473</v>
       </c>
       <c r="G7" t="n">
-        <v>738.1416666666668</v>
+        <v>-0.57000000000005</v>
       </c>
       <c r="H7" t="n">
-        <v>767.5916666666667</v>
+        <v>-0.09999999999990905</v>
       </c>
       <c r="I7" t="n">
-        <v>774.3366666666667</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>781.2883333333333</v>
+        <v>0.09999999999990905</v>
       </c>
       <c r="K7" t="n">
-        <v>817.875</v>
+        <v>0.7000000000000455</v>
       </c>
       <c r="L7" t="n">
-        <v>13.6966666666666</v>
+        <v>0.1999999999998181</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.2331679525960405</v>
+        <v>0.0734800260731755</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -1335,7 +1262,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>original</t>
+          <t>second_difference</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1364,34 +1291,34 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>14399</v>
+        <v>14400</v>
       </c>
       <c r="E8" t="n">
-        <v>774.063111558673</v>
+        <v>774.0630346064816</v>
       </c>
       <c r="F8" t="n">
-        <v>10.65469959781469</v>
+        <v>10.67342310535531</v>
       </c>
       <c r="G8" t="n">
-        <v>738.5908333333333</v>
+        <v>738.1416666666668</v>
       </c>
       <c r="H8" t="n">
-        <v>767.6266666666666</v>
+        <v>767.5916666666667</v>
       </c>
       <c r="I8" t="n">
-        <v>774.3191666666667</v>
+        <v>774.3366666666667</v>
       </c>
       <c r="J8" t="n">
-        <v>781.2629166666667</v>
+        <v>781.2883333333333</v>
       </c>
       <c r="K8" t="n">
-        <v>817.8216666666667</v>
+        <v>817.875</v>
       </c>
       <c r="L8" t="n">
-        <v>13.63625000000013</v>
+        <v>13.6966666666666</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.2348042247456309</v>
+        <v>-0.2331679525960405</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -1400,16 +1327,16 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>trailing_rolling_mean</t>
+          <t>original</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>1min</t>
+          <t>none</t>
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1429,34 +1356,34 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>14391</v>
+        <v>14399</v>
       </c>
       <c r="E9" t="n">
-        <v>774.0621507307809</v>
+        <v>774.063111558673</v>
       </c>
       <c r="F9" t="n">
-        <v>10.44579027278911</v>
+        <v>10.65469959781469</v>
       </c>
       <c r="G9" t="n">
-        <v>739.2941666666667</v>
+        <v>738.5908333333333</v>
       </c>
       <c r="H9" t="n">
-        <v>767.7525000000001</v>
+        <v>767.6266666666666</v>
       </c>
       <c r="I9" t="n">
-        <v>774.2688333333333</v>
+        <v>774.3191666666667</v>
       </c>
       <c r="J9" t="n">
-        <v>781.2188333333334</v>
+        <v>781.2629166666667</v>
       </c>
       <c r="K9" t="n">
-        <v>815.6681666666666</v>
+        <v>817.8216666666667</v>
       </c>
       <c r="L9" t="n">
-        <v>13.4663333333333</v>
+        <v>13.63625000000013</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.2477388017622714</v>
+        <v>-0.2348042247456309</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -1470,11 +1397,11 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>5min</t>
+          <t>1min</t>
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1494,34 +1421,34 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>14399</v>
+        <v>14391</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.0001983934069495578</v>
+        <v>774.0621507307809</v>
       </c>
       <c r="F10" t="n">
-        <v>1.275966503163818</v>
+        <v>10.44579027278911</v>
       </c>
       <c r="G10" t="n">
-        <v>-5.07000000000005</v>
+        <v>739.2941666666667</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.8441666666667516</v>
+        <v>767.7525000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.006666666666660603</v>
+        <v>774.2688333333333</v>
       </c>
       <c r="J10" t="n">
-        <v>0.839999999999975</v>
+        <v>781.2188333333334</v>
       </c>
       <c r="K10" t="n">
-        <v>6.251666666666551</v>
+        <v>815.6681666666666</v>
       </c>
       <c r="L10" t="n">
-        <v>1.684166666666727</v>
+        <v>13.4663333333333</v>
       </c>
       <c r="M10" t="n">
-        <v>0.01495842660680246</v>
+        <v>-0.2477388017622714</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -1530,16 +1457,16 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>first_difference</t>
+          <t>trailing_rolling_mean</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>5min</t>
         </is>
       </c>
       <c r="Q10" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -1559,34 +1486,34 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>14398</v>
+        <v>14399</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.0002175070611659023</v>
+        <v>-0.0001983934069495578</v>
       </c>
       <c r="F11" t="n">
-        <v>1.307370429648706</v>
+        <v>1.275966503163818</v>
       </c>
       <c r="G11" t="n">
-        <v>-5.708333333333371</v>
+        <v>-5.07000000000005</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.8599999999999852</v>
+        <v>-0.8441666666667516</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>-0.006666666666660603</v>
       </c>
       <c r="J11" t="n">
-        <v>0.8716666666667834</v>
+        <v>0.839999999999975</v>
       </c>
       <c r="K11" t="n">
-        <v>5.781666666666752</v>
+        <v>6.251666666666551</v>
       </c>
       <c r="L11" t="n">
-        <v>1.731666666666769</v>
+        <v>1.684166666666727</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.02177960641949485</v>
+        <v>0.01495842660680246</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -1595,7 +1522,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>second_difference</t>
+          <t>first_difference</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1610,12 +1537,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>subset_B_1min</t>
+          <t>subset_B_30s</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1min</t>
+          <t>30s</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1624,34 +1551,34 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>7200</v>
+        <v>14398</v>
       </c>
       <c r="E12" t="n">
-        <v>774.0630346064816</v>
+        <v>-0.0002175070611659023</v>
       </c>
       <c r="F12" t="n">
-        <v>10.65488860020091</v>
+        <v>1.307370429648706</v>
       </c>
       <c r="G12" t="n">
-        <v>738.5908333333333</v>
+        <v>-5.708333333333371</v>
       </c>
       <c r="H12" t="n">
-        <v>767.6404166666666</v>
+        <v>-0.8599999999999852</v>
       </c>
       <c r="I12" t="n">
-        <v>774.3362500000001</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>781.2702083333334</v>
+        <v>0.8716666666667834</v>
       </c>
       <c r="K12" t="n">
-        <v>817.8216666666667</v>
+        <v>5.781666666666752</v>
       </c>
       <c r="L12" t="n">
-        <v>13.62979166666673</v>
+        <v>1.731666666666769</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.2345766553598631</v>
+        <v>-0.02177960641949485</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -1660,7 +1587,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>original</t>
+          <t>second_difference</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1689,34 +1616,34 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>7196</v>
+        <v>7200</v>
       </c>
       <c r="E13" t="n">
-        <v>774.0622990087085</v>
+        <v>774.0630346064816</v>
       </c>
       <c r="F13" t="n">
-        <v>10.44590478279247</v>
+        <v>10.65488860020091</v>
       </c>
       <c r="G13" t="n">
-        <v>739.2941666666668</v>
+        <v>738.5908333333333</v>
       </c>
       <c r="H13" t="n">
-        <v>767.7795833333332</v>
+        <v>767.6404166666666</v>
       </c>
       <c r="I13" t="n">
-        <v>774.2785000000001</v>
+        <v>774.3362500000001</v>
       </c>
       <c r="J13" t="n">
-        <v>781.2075416666668</v>
+        <v>781.2702083333334</v>
       </c>
       <c r="K13" t="n">
-        <v>815.4731666666668</v>
+        <v>817.8216666666667</v>
       </c>
       <c r="L13" t="n">
-        <v>13.42795833333355</v>
+        <v>13.62979166666673</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.2477687711062135</v>
+        <v>-0.2345766553598631</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -1725,16 +1652,16 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>trailing_rolling_mean</t>
+          <t>original</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>5min</t>
+          <t>none</t>
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1754,34 +1681,34 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>7199</v>
+        <v>7196</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.0004478631291383016</v>
+        <v>774.0622990087085</v>
       </c>
       <c r="F14" t="n">
-        <v>2.016374070522469</v>
+        <v>10.44590478279247</v>
       </c>
       <c r="G14" t="n">
-        <v>-8.265833333333376</v>
+        <v>739.2941666666668</v>
       </c>
       <c r="H14" t="n">
-        <v>-1.320833333333269</v>
+        <v>767.7795833333332</v>
       </c>
       <c r="I14" t="n">
-        <v>0.01583333333337578</v>
+        <v>774.2785000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>1.327499999999986</v>
+        <v>781.2075416666668</v>
       </c>
       <c r="K14" t="n">
-        <v>9.15833333333353</v>
+        <v>815.4731666666668</v>
       </c>
       <c r="L14" t="n">
-        <v>2.648333333333255</v>
+        <v>13.42795833333355</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.01495259307717861</v>
+        <v>-0.2477687711062135</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -1790,16 +1717,16 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>first_difference</t>
+          <t>trailing_rolling_mean</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>5min</t>
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -1819,34 +1746,34 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7198</v>
+        <v>7199</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0005132212651662333</v>
+        <v>-0.0004478631291383016</v>
       </c>
       <c r="F15" t="n">
-        <v>2.309621217006801</v>
+        <v>2.016374070522469</v>
       </c>
       <c r="G15" t="n">
-        <v>-9.106666666666683</v>
+        <v>-8.265833333333376</v>
       </c>
       <c r="H15" t="n">
-        <v>-1.526875000000018</v>
+        <v>-1.320833333333269</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.01625000000001364</v>
+        <v>0.01583333333337578</v>
       </c>
       <c r="J15" t="n">
-        <v>1.572291666666757</v>
+        <v>1.327499999999986</v>
       </c>
       <c r="K15" t="n">
-        <v>12.26250000000016</v>
+        <v>9.15833333333353</v>
       </c>
       <c r="L15" t="n">
-        <v>3.099166666666775</v>
+        <v>2.648333333333255</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.006800918693741113</v>
+        <v>-0.01495259307717861</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -1855,7 +1782,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>second_difference</t>
+          <t>first_difference</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1870,12 +1797,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>subset_B_5min</t>
+          <t>subset_B_1min</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>5min</t>
+          <t>1min</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1884,34 +1811,34 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1440</v>
+        <v>7198</v>
       </c>
       <c r="E16" t="n">
-        <v>774.0630346064814</v>
+        <v>-0.0005132212651662333</v>
       </c>
       <c r="F16" t="n">
-        <v>10.44418514182298</v>
+        <v>2.309621217006801</v>
       </c>
       <c r="G16" t="n">
-        <v>739.5895</v>
+        <v>-9.106666666666683</v>
       </c>
       <c r="H16" t="n">
-        <v>767.8555</v>
+        <v>-1.526875000000018</v>
       </c>
       <c r="I16" t="n">
-        <v>774.2698333333333</v>
+        <v>-0.01625000000001364</v>
       </c>
       <c r="J16" t="n">
-        <v>781.1922916666667</v>
+        <v>1.572291666666757</v>
       </c>
       <c r="K16" t="n">
-        <v>815.4731666666667</v>
+        <v>12.26250000000016</v>
       </c>
       <c r="L16" t="n">
-        <v>13.33679166666673</v>
+        <v>3.099166666666775</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.2487446422150158</v>
+        <v>-0.006800918693741113</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -1920,7 +1847,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>original</t>
+          <t>second_difference</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1932,15 +1859,1105 @@
         <v>1</v>
       </c>
     </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id_key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>granularity</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>frequency</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>acf_30s</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>acf_1min</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>acf_5min</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>acf_10min</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5s</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>86400</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.9916661941774003</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.9773934132442712</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.8456591102333009</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.7160959422755356</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>14400</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9928528644568304</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.9789191558513288</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.8470592565397244</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.7173181952148976</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>7200</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9820925256559482</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.9820925256559482</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.8501700577102538</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.7200882547826742</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id_key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>granularity</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>transform</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>adf_statistic</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>adf_pvalue</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>adf_used_lag</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>adf_nobs</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>kpss_statistic</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>kpss_pvalue</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>kpss_used_lag</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>stationary_recommended</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>86400</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-11.59614553358569</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.717546204464789e-21</v>
+      </c>
+      <c r="G2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H2" t="n">
+        <v>86364</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.9859335453945668</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K2" t="n">
+        <v>171</v>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>first_difference</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>86399</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-84.37494449290195</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>86393</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.002386316442035272</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>102</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>second_difference</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>86398</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-55.69321961830641</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>66</v>
+      </c>
+      <c r="H4" t="n">
+        <v>86331</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.01487449827513698</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1751</v>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>14400</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-8.087124438337199</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.410039688905484e-12</v>
+      </c>
+      <c r="G5" t="n">
+        <v>25</v>
+      </c>
+      <c r="H5" t="n">
+        <v>14374</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.4536463392403571</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.05403175032743228</v>
+      </c>
+      <c r="K5" t="n">
+        <v>71</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>first_difference</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>14399</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-24.35863411902151</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>42</v>
+      </c>
+      <c r="H6" t="n">
+        <v>14356</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.003410636580385386</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>32</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>second_difference</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>14398</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-33.05549070761088</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>42</v>
+      </c>
+      <c r="H7" t="n">
+        <v>14355</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.01910025643267669</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>358</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>7200</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-6.738909717850945</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3.155324707751807e-09</v>
+      </c>
+      <c r="G8" t="n">
+        <v>21</v>
+      </c>
+      <c r="H8" t="n">
+        <v>7178</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.3382124415552797</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>51</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>first_difference</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>7199</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-23.7558413114052</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>22</v>
+      </c>
+      <c r="H9" t="n">
+        <v>7176</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.004385354410975745</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>23</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>second_difference</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>7198</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-26.52043278983831</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>35</v>
+      </c>
+      <c r="H10" t="n">
+        <v>7162</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.05793038162402646</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>626</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id_key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>granularity</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>target_column</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>variable</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>correlation</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>abs_correlation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ZZQBCHLL.AV_0#</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0.8686452093942587</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.8686452093942587</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>YFJ3_AI.AV_0#</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0.6519540110208691</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.6519540110208691</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TE_8319A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0.5843961325613678</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.5843961325613678</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TE_8303.AV_0#</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.3960038241581353</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.3960038241581353</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PTCA_8322A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.3933021289908426</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.3933021289908426</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AIR_8301A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.3836181603286373</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.3836181603286373</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TE_8332A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.3482625435659329</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.3482625435659329</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FT_8306A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>-0.1769908139033749</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.1769908139033749</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>FT_8301.AV_0#</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.1448947627458851</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.1448947627458851</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ZCLCCY.AV_0#</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0.1094947211607699</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.1094947211607699</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SXLTCYZ.AV_0#</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0.0918766061566712</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.0918766061566712</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PT_8313C.AV_0#</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0.07239954271005011</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.07239954271005011</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>YFJ3_ZD2.AV_0#</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>-0.02149552245792387</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.02149552245792387</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ZZQBCHLL.AV_0#</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0.8718777539515006</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.8718777539515006</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>YFJ3_AI.AV_0#</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0.7418477682984967</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.7418477682984967</v>
+      </c>
+    </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>subset_B_5min</t>
+          <t>subset_B_30s</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>5min</t>
+          <t>30s</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1948,64 +2965,27 @@
           <t>TE_8313B.AV_0#</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>1439</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>TE_8319A.AV_0#</t>
+        </is>
       </c>
       <c r="E17" t="n">
-        <v>-0.005517373175816506</v>
+        <v>0.5848451746697336</v>
       </c>
       <c r="F17" t="n">
-        <v>4.930875634963402</v>
-      </c>
-      <c r="G17" t="n">
-        <v>-21.16183333333333</v>
-      </c>
-      <c r="H17" t="n">
-        <v>-3.032000000000039</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0.04066666666665242</v>
-      </c>
-      <c r="J17" t="n">
-        <v>2.968083333333311</v>
-      </c>
-      <c r="K17" t="n">
-        <v>23.65350000000001</v>
-      </c>
-      <c r="L17" t="n">
-        <v>6.00008333333335</v>
-      </c>
-      <c r="M17" t="n">
-        <v>-0.01881392495967665</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>TE_8313B.AV_0#</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>first_difference</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="Q17" t="n">
-        <v>1</v>
+        <v>0.5848451746697336</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>subset_B_5min</t>
+          <t>subset_B_30s</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>5min</t>
+          <t>30s</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2013,53 +2993,632 @@
           <t>TE_8313B.AV_0#</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>1438</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>TE_8303.AV_0#</t>
+        </is>
       </c>
       <c r="E18" t="n">
-        <v>0.0008157162726008358</v>
+        <v>0.3963346509390027</v>
       </c>
       <c r="F18" t="n">
-        <v>6.647188052345607</v>
-      </c>
-      <c r="G18" t="n">
-        <v>-38.55183333333332</v>
-      </c>
-      <c r="H18" t="n">
-        <v>-4.078541666666865</v>
-      </c>
-      <c r="I18" t="n">
-        <v>-0.2574166666666429</v>
-      </c>
-      <c r="J18" t="n">
-        <v>3.837124999999929</v>
-      </c>
-      <c r="K18" t="n">
-        <v>26.7788333333333</v>
-      </c>
-      <c r="L18" t="n">
-        <v>7.915666666666795</v>
-      </c>
-      <c r="M18" t="n">
-        <v>-0.03192289816668104</v>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>TE_8313B.AV_0#</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>second_difference</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="Q18" t="n">
-        <v>1</v>
+        <v>0.3963346509390027</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>PTCA_8322A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0.394047364573897</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.394047364573897</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>AIR_8301A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>-0.3850427486536755</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.3850427486536755</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>TE_8332A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0.3484826351054031</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.3484826351054031</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>FT_8306A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>-0.1824454347462013</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.1824454347462013</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>FT_8301.AV_0#</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0.1532166734710194</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.1532166734710194</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ZCLCCY.AV_0#</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0.1109686100164222</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.1109686100164222</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>SXLTCYZ.AV_0#</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0.09322624469635216</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.09322624469635216</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>PT_8313C.AV_0#</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.07355928174308193</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.07355928174308193</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>YFJ3_ZD2.AV_0#</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>-0.04133120305222042</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.04133120305222042</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ZZQBCHLL.AV_0#</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0.8766784228124077</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.8766784228124077</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>YFJ3_AI.AV_0#</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0.7514155110192929</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.7514155110192929</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>TE_8319A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0.5857980634467633</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.5857980634467633</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>TE_8303.AV_0#</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0.3970635878785198</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.3970635878785198</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>PTCA_8322A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0.3949267041377826</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.3949267041377826</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>AIR_8301A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>-0.3873087894703714</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.3873087894703714</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>TE_8332A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0.3488976490980261</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.3488976490980261</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>FT_8306A.AV_0#</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>-0.1836438459873214</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.1836438459873214</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>FT_8301.AV_0#</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0.1548245008727568</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.1548245008727568</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>ZCLCCY.AV_0#</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0.11121432165591</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.11121432165591</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>SXLTCYZ.AV_0#</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0.09442459159841289</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.09442459159841289</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>PT_8313C.AV_0#</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0.07479054814297063</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.07479054814297063</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>YFJ3_ZD2.AV_0#</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>-0.04858174837161518</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.04858174837161518</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor forecasting candidate review workflow
- Remove validation-based MLP selection and use chronological train/test only
- Add raw dataset to univariate candidate review
- Update smoothing candidates by granularity and remove 5min smoothing
- Add R2 to forecasting metrics and reports
- Switch MLP training from sklearn to NeuralForecast MLP
- Configure one-step MLP horizon for assignment stage
- Add learning-rate grid with 0.005 and min/max training steps
- Enable GPU-backed NeuralForecast training configuration
- Update forecasting plots/reports for per-candidate test comparison
- Add VS Code debug launch configs for orchestrator runs
</commit_message>
<xml_diff>
--- a/outputs/chinese_boiler_dataset/tables/pre_forecasting_summary.xlsx
+++ b/outputs/chinese_boiler_dataset/tables/pre_forecasting_summary.xlsx
@@ -794,7 +794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -966,34 +966,34 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>86395</v>
+        <v>86398</v>
       </c>
       <c r="E3" t="n">
-        <v>774.0631044427726</v>
+        <v>774.0630618764324</v>
       </c>
       <c r="F3" t="n">
-        <v>10.67337210764209</v>
+        <v>10.67958164355307</v>
       </c>
       <c r="G3" t="n">
-        <v>738.0649999999999</v>
+        <v>737.79</v>
       </c>
       <c r="H3" t="n">
-        <v>767.5983333333334</v>
+        <v>767.59</v>
       </c>
       <c r="I3" t="n">
-        <v>774.3250000000002</v>
+        <v>774.3200000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>781.275</v>
+        <v>781.2766666666666</v>
       </c>
       <c r="K3" t="n">
-        <v>818.0116666666667</v>
+        <v>818.08</v>
       </c>
       <c r="L3" t="n">
-        <v>13.67666666666662</v>
+        <v>13.68666666666661</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.2331823403697795</v>
+        <v>-0.2325990379527573</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -1007,11 +1007,11 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>30s</t>
+          <t>15s</t>
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -1031,34 +1031,34 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>86389</v>
+        <v>86395</v>
       </c>
       <c r="E4" t="n">
-        <v>774.0631438319693</v>
+        <v>774.0631044427726</v>
       </c>
       <c r="F4" t="n">
-        <v>10.65468342157003</v>
+        <v>10.67337210764209</v>
       </c>
       <c r="G4" t="n">
-        <v>738.5091666666667</v>
+        <v>738.0649999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>767.6083333333335</v>
+        <v>767.5983333333334</v>
       </c>
       <c r="I4" t="n">
-        <v>774.3366666666667</v>
+        <v>774.3250000000002</v>
       </c>
       <c r="J4" t="n">
-        <v>781.2675</v>
+        <v>781.275</v>
       </c>
       <c r="K4" t="n">
-        <v>817.8891666666667</v>
+        <v>818.0116666666667</v>
       </c>
       <c r="L4" t="n">
-        <v>13.65916666666658</v>
+        <v>13.67666666666662</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.2347992594581003</v>
+        <v>-0.2331823403697795</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -1072,11 +1072,11 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>1min</t>
+          <t>30s</t>
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -1096,34 +1096,34 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>86341</v>
+        <v>86389</v>
       </c>
       <c r="E5" t="n">
-        <v>774.0620165989121</v>
+        <v>774.0631438319693</v>
       </c>
       <c r="F5" t="n">
-        <v>10.44573072329733</v>
+        <v>10.65468342157003</v>
       </c>
       <c r="G5" t="n">
-        <v>739.2755</v>
+        <v>738.5091666666667</v>
       </c>
       <c r="H5" t="n">
-        <v>767.7516666666667</v>
+        <v>767.6083333333335</v>
       </c>
       <c r="I5" t="n">
-        <v>774.2495</v>
+        <v>774.3366666666667</v>
       </c>
       <c r="J5" t="n">
-        <v>781.2196666666666</v>
+        <v>781.2675</v>
       </c>
       <c r="K5" t="n">
-        <v>815.6681666666666</v>
+        <v>817.8891666666667</v>
       </c>
       <c r="L5" t="n">
-        <v>13.46799999999996</v>
+        <v>13.65916666666658</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.2476865316551196</v>
+        <v>-0.2347992594581003</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -1137,11 +1137,11 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>5min</t>
+          <t>1min</t>
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -1161,34 +1161,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>86399</v>
+        <v>86377</v>
       </c>
       <c r="E6" t="n">
-        <v>-2.673642056042384e-05</v>
+        <v>774.063057034859</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2732205123091537</v>
+        <v>10.60776935268142</v>
       </c>
       <c r="G6" t="n">
-        <v>-1.139999999999986</v>
+        <v>738.6929166666665</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.1700000000000728</v>
+        <v>767.6525</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>774.3170833333334</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1700000000000728</v>
+        <v>781.2829166666666</v>
       </c>
       <c r="K6" t="n">
-        <v>1.299999999999955</v>
+        <v>817.4841666666666</v>
       </c>
       <c r="L6" t="n">
-        <v>0.3400000000001455</v>
+        <v>13.63041666666652</v>
       </c>
       <c r="M6" t="n">
-        <v>0.03859649943443079</v>
+        <v>-0.2383367291790616</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -1197,16 +1197,16 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>first_difference</t>
+          <t>trailing_rolling_mean</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>2min</t>
         </is>
       </c>
       <c r="Q6" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -1226,34 +1226,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>86398</v>
+        <v>86365</v>
       </c>
       <c r="E7" t="n">
-        <v>2.777842079677876e-06</v>
+        <v>774.062810761175</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1383208577587473</v>
+        <v>10.55637588497761</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.57000000000005</v>
+        <v>738.8875</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.09999999999990905</v>
+        <v>767.6894444444445</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>774.3016666666667</v>
       </c>
       <c r="J7" t="n">
-        <v>0.09999999999990905</v>
+        <v>781.2538888888889</v>
       </c>
       <c r="K7" t="n">
-        <v>0.7000000000000455</v>
+        <v>816.6136111111111</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1999999999998181</v>
+        <v>13.56444444444446</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0734800260731755</v>
+        <v>-0.2416162363927248</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -1262,27 +1262,27 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>second_difference</t>
+          <t>trailing_rolling_mean</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>3min</t>
         </is>
       </c>
       <c r="Q7" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>subset_B_30s</t>
+          <t>subset_B_raw</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>30s</t>
+          <t>raw</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1291,34 +1291,34 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>14400</v>
+        <v>86399</v>
       </c>
       <c r="E8" t="n">
-        <v>774.0630346064816</v>
+        <v>-2.673642056042384e-05</v>
       </c>
       <c r="F8" t="n">
-        <v>10.67342310535531</v>
+        <v>0.2732205123091537</v>
       </c>
       <c r="G8" t="n">
-        <v>738.1416666666668</v>
+        <v>-1.139999999999986</v>
       </c>
       <c r="H8" t="n">
-        <v>767.5916666666667</v>
+        <v>-0.1700000000000728</v>
       </c>
       <c r="I8" t="n">
-        <v>774.3366666666667</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>781.2883333333333</v>
+        <v>0.1700000000000728</v>
       </c>
       <c r="K8" t="n">
-        <v>817.875</v>
+        <v>1.299999999999955</v>
       </c>
       <c r="L8" t="n">
-        <v>13.6966666666666</v>
+        <v>0.3400000000001455</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.2331679525960405</v>
+        <v>0.03859649943443079</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>original</t>
+          <t>first_difference</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1342,12 +1342,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>subset_B_30s</t>
+          <t>subset_B_raw</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>30s</t>
+          <t>raw</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1356,34 +1356,34 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>14399</v>
+        <v>86398</v>
       </c>
       <c r="E9" t="n">
-        <v>774.063111558673</v>
+        <v>2.777842079677876e-06</v>
       </c>
       <c r="F9" t="n">
-        <v>10.65469959781469</v>
+        <v>0.1383208577587473</v>
       </c>
       <c r="G9" t="n">
-        <v>738.5908333333333</v>
+        <v>-0.57000000000005</v>
       </c>
       <c r="H9" t="n">
-        <v>767.6266666666666</v>
+        <v>-0.09999999999990905</v>
       </c>
       <c r="I9" t="n">
-        <v>774.3191666666667</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>781.2629166666667</v>
+        <v>0.09999999999990905</v>
       </c>
       <c r="K9" t="n">
-        <v>817.8216666666667</v>
+        <v>0.7000000000000455</v>
       </c>
       <c r="L9" t="n">
-        <v>13.63625000000013</v>
+        <v>0.1999999999998181</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.2348042247456309</v>
+        <v>0.0734800260731755</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -1392,16 +1392,16 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>trailing_rolling_mean</t>
+          <t>second_difference</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>1min</t>
+          <t>none</t>
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1421,34 +1421,34 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>14391</v>
+        <v>14400</v>
       </c>
       <c r="E10" t="n">
-        <v>774.0621507307809</v>
+        <v>774.0630346064816</v>
       </c>
       <c r="F10" t="n">
-        <v>10.44579027278911</v>
+        <v>10.67342310535531</v>
       </c>
       <c r="G10" t="n">
-        <v>739.2941666666667</v>
+        <v>738.1416666666668</v>
       </c>
       <c r="H10" t="n">
-        <v>767.7525000000001</v>
+        <v>767.5916666666667</v>
       </c>
       <c r="I10" t="n">
-        <v>774.2688333333333</v>
+        <v>774.3366666666667</v>
       </c>
       <c r="J10" t="n">
-        <v>781.2188333333334</v>
+        <v>781.2883333333333</v>
       </c>
       <c r="K10" t="n">
-        <v>815.6681666666666</v>
+        <v>817.875</v>
       </c>
       <c r="L10" t="n">
-        <v>13.4663333333333</v>
+        <v>13.6966666666666</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.2477388017622714</v>
+        <v>-0.2331679525960405</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -1457,16 +1457,16 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>trailing_rolling_mean</t>
+          <t>original</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>5min</t>
+          <t>none</t>
         </is>
       </c>
       <c r="Q10" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1489,31 +1489,31 @@
         <v>14399</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.0001983934069495578</v>
+        <v>774.063111558673</v>
       </c>
       <c r="F11" t="n">
-        <v>1.275966503163818</v>
+        <v>10.65469959781469</v>
       </c>
       <c r="G11" t="n">
-        <v>-5.07000000000005</v>
+        <v>738.5908333333333</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.8441666666667516</v>
+        <v>767.6266666666666</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.006666666666660603</v>
+        <v>774.3191666666667</v>
       </c>
       <c r="J11" t="n">
-        <v>0.839999999999975</v>
+        <v>781.2629166666667</v>
       </c>
       <c r="K11" t="n">
-        <v>6.251666666666551</v>
+        <v>817.8216666666667</v>
       </c>
       <c r="L11" t="n">
-        <v>1.684166666666727</v>
+        <v>13.63625000000013</v>
       </c>
       <c r="M11" t="n">
-        <v>0.01495842660680246</v>
+        <v>-0.2348042247456309</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -1522,16 +1522,16 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>first_difference</t>
+          <t>trailing_rolling_mean</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>1min</t>
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -1551,34 +1551,34 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>14398</v>
+        <v>14397</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.0002175070611659023</v>
+        <v>774.0630810527657</v>
       </c>
       <c r="F12" t="n">
-        <v>1.307370429648706</v>
+        <v>10.60778417021666</v>
       </c>
       <c r="G12" t="n">
-        <v>-5.708333333333371</v>
+        <v>738.7758333333334</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.8599999999999852</v>
+        <v>767.6495833333333</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>774.3266666666666</v>
       </c>
       <c r="J12" t="n">
-        <v>0.8716666666667834</v>
+        <v>781.3000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>5.781666666666752</v>
+        <v>817.4383333333333</v>
       </c>
       <c r="L12" t="n">
-        <v>1.731666666666769</v>
+        <v>13.65041666666673</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.02177960641949485</v>
+        <v>-0.2383621969096129</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -1587,27 +1587,27 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>second_difference</t>
+          <t>trailing_rolling_mean</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>2min</t>
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>subset_B_1min</t>
+          <t>subset_B_30s</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1min</t>
+          <t>30s</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1616,34 +1616,34 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>7200</v>
+        <v>14395</v>
       </c>
       <c r="E13" t="n">
-        <v>774.0630346064816</v>
+        <v>774.062887113581</v>
       </c>
       <c r="F13" t="n">
-        <v>10.65488860020091</v>
+        <v>10.55640369928853</v>
       </c>
       <c r="G13" t="n">
-        <v>738.5908333333333</v>
+        <v>738.9077777777778</v>
       </c>
       <c r="H13" t="n">
-        <v>767.6404166666666</v>
+        <v>767.6870833333332</v>
       </c>
       <c r="I13" t="n">
-        <v>774.3362500000001</v>
+        <v>774.3083333333334</v>
       </c>
       <c r="J13" t="n">
-        <v>781.2702083333334</v>
+        <v>781.2694444444444</v>
       </c>
       <c r="K13" t="n">
-        <v>817.8216666666667</v>
+        <v>816.613611111111</v>
       </c>
       <c r="L13" t="n">
-        <v>13.62979166666673</v>
+        <v>13.58236111111114</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.2345766553598631</v>
+        <v>-0.2416553691084035</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -1652,27 +1652,27 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>original</t>
+          <t>trailing_rolling_mean</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>3min</t>
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>subset_B_1min</t>
+          <t>subset_B_30s</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1min</t>
+          <t>30s</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1681,34 +1681,34 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>7196</v>
+        <v>14399</v>
       </c>
       <c r="E14" t="n">
-        <v>774.0622990087085</v>
+        <v>-0.0001983934069495578</v>
       </c>
       <c r="F14" t="n">
-        <v>10.44590478279247</v>
+        <v>1.275966503163818</v>
       </c>
       <c r="G14" t="n">
-        <v>739.2941666666668</v>
+        <v>-5.07000000000005</v>
       </c>
       <c r="H14" t="n">
-        <v>767.7795833333332</v>
+        <v>-0.8441666666667516</v>
       </c>
       <c r="I14" t="n">
-        <v>774.2785000000001</v>
+        <v>-0.006666666666660603</v>
       </c>
       <c r="J14" t="n">
-        <v>781.2075416666668</v>
+        <v>0.839999999999975</v>
       </c>
       <c r="K14" t="n">
-        <v>815.4731666666668</v>
+        <v>6.251666666666551</v>
       </c>
       <c r="L14" t="n">
-        <v>13.42795833333355</v>
+        <v>1.684166666666727</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.2477687711062135</v>
+        <v>0.01495842660680246</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -1717,27 +1717,27 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>trailing_rolling_mean</t>
+          <t>first_difference</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>5min</t>
+          <t>none</t>
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>subset_B_1min</t>
+          <t>subset_B_30s</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1min</t>
+          <t>30s</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1746,34 +1746,34 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7199</v>
+        <v>14398</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0004478631291383016</v>
+        <v>-0.0002175070611659023</v>
       </c>
       <c r="F15" t="n">
-        <v>2.016374070522469</v>
+        <v>1.307370429648706</v>
       </c>
       <c r="G15" t="n">
-        <v>-8.265833333333376</v>
+        <v>-5.708333333333371</v>
       </c>
       <c r="H15" t="n">
-        <v>-1.320833333333269</v>
+        <v>-0.8599999999999852</v>
       </c>
       <c r="I15" t="n">
-        <v>0.01583333333337578</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>1.327499999999986</v>
+        <v>0.8716666666667834</v>
       </c>
       <c r="K15" t="n">
-        <v>9.15833333333353</v>
+        <v>5.781666666666752</v>
       </c>
       <c r="L15" t="n">
-        <v>2.648333333333255</v>
+        <v>1.731666666666769</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.01495259307717861</v>
+        <v>-0.02177960641949485</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>first_difference</t>
+          <t>second_difference</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1811,51 +1811,311 @@
         </is>
       </c>
       <c r="D16" t="n">
+        <v>7200</v>
+      </c>
+      <c r="E16" t="n">
+        <v>774.0630346064816</v>
+      </c>
+      <c r="F16" t="n">
+        <v>10.65488860020091</v>
+      </c>
+      <c r="G16" t="n">
+        <v>738.5908333333333</v>
+      </c>
+      <c r="H16" t="n">
+        <v>767.6404166666666</v>
+      </c>
+      <c r="I16" t="n">
+        <v>774.3362500000001</v>
+      </c>
+      <c r="J16" t="n">
+        <v>781.2702083333334</v>
+      </c>
+      <c r="K16" t="n">
+        <v>817.8216666666667</v>
+      </c>
+      <c r="L16" t="n">
+        <v>13.62979166666673</v>
+      </c>
+      <c r="M16" t="n">
+        <v>-0.2345766553598631</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>7199</v>
+      </c>
+      <c r="E17" t="n">
+        <v>774.0630797680234</v>
+      </c>
+      <c r="F17" t="n">
+        <v>10.60780873567199</v>
+      </c>
+      <c r="G17" t="n">
+        <v>738.8699999999999</v>
+      </c>
+      <c r="H17" t="n">
+        <v>767.6522916666667</v>
+      </c>
+      <c r="I17" t="n">
+        <v>774.2950000000001</v>
+      </c>
+      <c r="J17" t="n">
+        <v>781.2887499999999</v>
+      </c>
+      <c r="K17" t="n">
+        <v>817.4383333333333</v>
+      </c>
+      <c r="L17" t="n">
+        <v>13.63645833333328</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-0.2382941219093036</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>2min</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
         <v>7198</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E18" t="n">
+        <v>774.0629538683586</v>
+      </c>
+      <c r="F18" t="n">
+        <v>10.55647320854445</v>
+      </c>
+      <c r="G18" t="n">
+        <v>738.9077777777778</v>
+      </c>
+      <c r="H18" t="n">
+        <v>767.6925</v>
+      </c>
+      <c r="I18" t="n">
+        <v>774.3120833333332</v>
+      </c>
+      <c r="J18" t="n">
+        <v>781.2721527777778</v>
+      </c>
+      <c r="K18" t="n">
+        <v>816.3416666666667</v>
+      </c>
+      <c r="L18" t="n">
+        <v>13.57965277777782</v>
+      </c>
+      <c r="M18" t="n">
+        <v>-0.2416512443019944</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>3min</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>7199</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-0.0004478631291383016</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2.016374070522469</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-8.265833333333376</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-1.320833333333269</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.01583333333337578</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1.327499999999986</v>
+      </c>
+      <c r="K19" t="n">
+        <v>9.15833333333353</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2.648333333333255</v>
+      </c>
+      <c r="M19" t="n">
+        <v>-0.01495259307717861</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>first_difference</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>7198</v>
+      </c>
+      <c r="E20" t="n">
         <v>-0.0005132212651662333</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F20" t="n">
         <v>2.309621217006801</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G20" t="n">
         <v>-9.106666666666683</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H20" t="n">
         <v>-1.526875000000018</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I20" t="n">
         <v>-0.01625000000001364</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J20" t="n">
         <v>1.572291666666757</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K20" t="n">
         <v>12.26250000000016</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L20" t="n">
         <v>3.099166666666775</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M20" t="n">
         <v>-0.006800918693741113</v>
       </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>TE_8313B.AV_0#</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
         <is>
           <t>second_difference</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="Q16" t="n">
+      <c r="Q20" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor MLP candidate review and document selected setup
- Switch MLP candidate review to chronological test-block comparison
- Use standard scaling after minmax vs z-score diagnostics
- Add scaler comparison plots, tables, and report rationale
- Run and archive full one-step MLP candidate review
- Remove duplicate/stale current forecasting summary artifacts
- Clarify ARIMA result naming while ARIMA remains disabled
- Add selected MLP candidate combinations for next-stage runs
- Add candidate selection report with metric, smoothing, transform, and LR evidence
- Add MLP progress logging, smoke-test controls, and run duration metadata
- Keep local history archives ignored by Git
</commit_message>
<xml_diff>
--- a/outputs/chinese_boiler_dataset/tables/pre_forecasting_summary.xlsx
+++ b/outputs/chinese_boiler_dataset/tables/pre_forecasting_summary.xlsx
@@ -10,9 +10,10 @@
     <sheet name="granularity" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="target_distribution" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="target_transforms" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="target_autocorrelation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="target_stationarity" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="target_correlations" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="target_scaling_comparison" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="target_autocorrelation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="target_stationarity" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="target_correlations" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -794,7 +795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -883,6 +884,11 @@
           <t>window_steps</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>scaling_method</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -948,6 +954,11 @@
       <c r="Q2" t="n">
         <v>1</v>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1013,6 +1024,11 @@
       <c r="Q3" t="n">
         <v>3</v>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1078,6 +1094,11 @@
       <c r="Q4" t="n">
         <v>6</v>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1143,6 +1164,11 @@
       <c r="Q5" t="n">
         <v>12</v>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1208,6 +1234,11 @@
       <c r="Q6" t="n">
         <v>24</v>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1273,6 +1304,11 @@
       <c r="Q7" t="n">
         <v>36</v>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1338,6 +1374,11 @@
       <c r="Q8" t="n">
         <v>1</v>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1403,6 +1444,11 @@
       <c r="Q9" t="n">
         <v>1</v>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1468,6 +1514,11 @@
       <c r="Q10" t="n">
         <v>1</v>
       </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1533,6 +1584,11 @@
       <c r="Q11" t="n">
         <v>2</v>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1598,6 +1654,11 @@
       <c r="Q12" t="n">
         <v>4</v>
       </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1663,6 +1724,11 @@
       <c r="Q13" t="n">
         <v>6</v>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1728,6 +1794,11 @@
       <c r="Q14" t="n">
         <v>1</v>
       </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1793,6 +1864,11 @@
       <c r="Q15" t="n">
         <v>1</v>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1858,6 +1934,11 @@
       <c r="Q16" t="n">
         <v>1</v>
       </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1923,6 +2004,11 @@
       <c r="Q17" t="n">
         <v>2</v>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1988,6 +2074,11 @@
       <c r="Q18" t="n">
         <v>3</v>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2053,6 +2144,11 @@
       <c r="Q19" t="n">
         <v>1</v>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2117,6 +2213,11 @@
       </c>
       <c r="Q20" t="n">
         <v>1</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>unscaled</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2130,7 +2231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:R39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2146,32 +2247,82 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>frequency</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>rows</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>acf_30s</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>acf_1min</t>
+          <t>std</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>acf_5min</t>
+          <t>min</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>acf_10min</t>
+          <t>q1</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>median</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>q3</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>iqr</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>skewness</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>transform</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>window</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>window_steps</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>scaling_method</t>
         </is>
       </c>
     </row>
@@ -2188,87 +2339,2651 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>5s</t>
+          <t>TE_8313B.AV_0#</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>86400</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9916661941774003</v>
+        <v>0.5537236882363554</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9773934132442712</v>
+        <v>0.1626570937498321</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8456591102333009</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0.7160959422755356</v>
+        <v>0.4551545606821989</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.5576366681894325</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.6636211359829444</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1.223998781787727</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.2084665753007454</v>
+      </c>
+      <c r="M2" t="n">
+        <v>-0.2323882392172661</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>scaled_level</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>subset_B_30s</t>
+          <t>subset_B_raw</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>30s</t>
+          <t>raw</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>30s</t>
+          <t>TE_8313B.AV_0#</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>14400</v>
+        <v>86398</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9928528644568304</v>
+        <v>0.5537241034937155</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9789191558513288</v>
+        <v>0.1626249679237563</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8470592565397244</v>
+        <v>0.001370488807673884</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7173181952148976</v>
+        <v>0.4551545606821982</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.5576366681894314</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.6635703771382161</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1.223998781787727</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.2084158164560179</v>
+      </c>
+      <c r="M3" t="n">
+        <v>-0.2325990379527492</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>15s</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>3</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>86395</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.5537247516791917</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1625304112630135</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.005558093497791267</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.45528145779402</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.5577128064565248</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.6635449977158516</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1.222958225470788</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.2082635399218316</v>
+      </c>
+      <c r="M4" t="n">
+        <v>-0.2331823403697751</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>86389</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.5537253514842291</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.162245826428659</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.01232170955788965</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.4554337343282062</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.5578904624130751</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.6634307903152123</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1.221092837927009</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.2079970559870061</v>
+      </c>
+      <c r="M5" t="n">
+        <v>-0.2347992594581016</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>12</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>86377</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.5537240297679122</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.1615314352471665</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.01511979087355889</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.4561062890208616</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.5575922542002939</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.6636655499720823</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1.214925638292472</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.2075592609512207</v>
+      </c>
+      <c r="M6" t="n">
+        <v>-0.238336729179023</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>2min</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>24</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>86365</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.5537202795976107</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.1607488333329924</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.01808283843459652</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.4566688662166045</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.5573574945434239</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.6632235250325701</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1.201669120010828</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.2065546588159656</v>
+      </c>
+      <c r="M7" t="n">
+        <v>-0.2416162363927585</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>3min</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>36</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>86399</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-4.071329459482857e-07</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.004160507268298369</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-0.01735952489721315</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-0.002588701081164491</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.002588701081164491</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.01979594944418994</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.005177402162328981</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.03859649943443094</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>scaled_first_difference</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>86398</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.230001644096012e-08</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.002106302082514807</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-0.008679762448607464</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-0.001522765341859467</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.001522765341859356</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.01065935739302648</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.003045530683718822</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.07348002607317548</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>scaled_second_difference</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>1</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>86400</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.09196513412658387</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.9948336943886197</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-3.294686930897382</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-0.5108975327066343</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.1158974706330712</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.7641134027644663</v>
+      </c>
+      <c r="K10" t="n">
+        <v>4.191462009436255</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1.275010935471101</v>
+      </c>
+      <c r="M10" t="n">
+        <v>-0.2323882392172655</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>scaled_level</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>86398</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.09196767389908532</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.9946372083116619</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-3.286304828326722</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-0.5108975327066377</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.1158974706330665</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.7638029545211129</v>
+      </c>
+      <c r="K11" t="n">
+        <v>4.191462009436255</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1.274700487227751</v>
+      </c>
+      <c r="M11" t="n">
+        <v>-0.2325990379527481</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>15s</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>3</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>86395</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.09197163829274821</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.9940588864569723</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-3.260692848249691</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-0.5101214120982436</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.1163631429981043</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.7636477303994316</v>
+      </c>
+      <c r="K12" t="n">
+        <v>4.185097820447414</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1.273769142497675</v>
+      </c>
+      <c r="M12" t="n">
+        <v>-0.2331823403697744</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>6</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>86389</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.09197530678483541</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.9923183255284506</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-3.219325619822244</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-0.5091900673681687</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.1174497118498562</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.7629492218518776</v>
+      </c>
+      <c r="K13" t="n">
+        <v>4.173688847504008</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1.272139289220046</v>
+      </c>
+      <c r="M13" t="n">
+        <v>-0.2347992594581022</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>12</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>86377</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.09196722298168737</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.9879490084458775</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-3.202212160407138</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-0.5050766281436753</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.1156258284201279</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.7643850449774064</v>
+      </c>
+      <c r="K14" t="n">
+        <v>4.135969385936018</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1.269461673121082</v>
+      </c>
+      <c r="M14" t="n">
+        <v>-0.2383367291790219</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>2min</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>24</v>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>86365</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.09194428641194032</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.983162504915261</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-3.184089744201117</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-0.5016358267797916</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.1141900052945978</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.7616815581914984</v>
+      </c>
+      <c r="K15" t="n">
+        <v>4.0548906530457</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1.26331738497129</v>
+      </c>
+      <c r="M15" t="n">
+        <v>-0.2416162363927575</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>3min</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
+        <v>36</v>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>86399</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-2.490082438998909e-06</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.02544624842872088</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-0.1061732992284181</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-0.01583286041126231</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.01583286041126229</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.1210748149095968</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.0316657208225246</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.03859649943443084</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>scaled_first_difference</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>86398</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2.587128581885368e-07</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.01288244019329044</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-0.0530866496142145</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-0.009313447300730082</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.009313447300729916</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.06519413110517402</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.01862689460146</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.07348002607317557</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>scaled_second_difference</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>1</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>14400</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.5548558532563296</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.1648659732059828</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.4548965091133763</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.5590824837812789</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.6664607146534852</v>
+      </c>
+      <c r="K18" t="n">
+        <v>1.231593038821955</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.211564205540109</v>
+      </c>
+      <c r="M18" t="n">
+        <v>-0.2331679525960218</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>scaled_level</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>1</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>14399</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.5548570418907374</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.1645767624005978</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.006938008444030077</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.4554371331479752</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.5588121717639777</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.6660681186283589</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1.230769230769231</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.2106309854803837</v>
+      </c>
+      <c r="M19" t="n">
+        <v>-0.2348042247456559</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>2</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>14397</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.5548565706842588</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.1638520878933686</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.009795592626916497</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.4557911131706306</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.5589280197713928</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.6666409226650196</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1.22484811039028</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.210849809494389</v>
+      </c>
+      <c r="M20" t="n">
+        <v>-0.2383621969095871</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>2min</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
+        <v>4</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>14395</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.5548535750218473</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.1630584445364311</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.01183365942401949</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.4563703532077021</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.558644835753269</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.6661689493014787</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1.212109120241651</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.2097985960937766</v>
+      </c>
+      <c r="M21" t="n">
+        <v>-0.2416553691084205</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>3min</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
+        <v>6</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>14399</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-3.064464117231358e-06</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.01970909025585141</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-0.07831325301204917</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-0.01303933683451886</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-0.0001029760065903718</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.01297497683039814</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.09656575018020636</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.02601431366491699</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.01495842660680267</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>scaled_first_difference</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
+        <v>1</v>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>14398</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-3.359701284613878e-06</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.02019416789695255</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-0.08817320564308595</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-0.01328390485016967</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.01346411286170501</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0.0893059417155817</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.02674801771187468</v>
+      </c>
+      <c r="M23" t="n">
+        <v>-0.02177960641949482</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>scaled_second_difference</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>1</v>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>14400</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.09203832181785054</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.9948547318058244</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-3.256141780770997</v>
+      </c>
+      <c r="H24" t="n">
+        <v>-0.511148767519121</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.1175431806772782</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.7654982377385986</v>
+      </c>
+      <c r="K24" t="n">
+        <v>4.175689897438956</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1.27664700525772</v>
+      </c>
+      <c r="M24" t="n">
+        <v>-0.2331679525960215</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>scaled_level</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>1</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>14399</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.09204549442322141</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.9931095400441069</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-3.214275588520224</v>
+      </c>
+      <c r="H25" t="n">
+        <v>-0.5078864668242611</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.1159120303298385</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.7631291860435139</v>
+      </c>
+      <c r="K25" t="n">
+        <v>4.170718772570585</v>
+      </c>
+      <c r="L25" t="n">
+        <v>1.271015652867775</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-0.2348042247456556</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>2</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>14397</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.0920426510105654</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.9887366191283075</v>
+      </c>
+      <c r="G26" t="n">
+        <v>-3.197031999133069</v>
+      </c>
+      <c r="H26" t="n">
+        <v>-0.5057504366073802</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.116611094764457</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.7665856713035606</v>
+      </c>
+      <c r="K26" t="n">
+        <v>4.134988812579194</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1.272336107910941</v>
+      </c>
+      <c r="M26" t="n">
+        <v>-0.2383621969095882</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>2min</t>
+        </is>
+      </c>
+      <c r="Q26" t="n">
+        <v>4</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>14395</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.09202457421238244</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.9839475178136959</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-3.184733643338929</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-0.5022551144343076</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.1149022705909552</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.763737631014384</v>
+      </c>
+      <c r="K27" t="n">
+        <v>4.058117616046984</v>
+      </c>
+      <c r="L27" t="n">
+        <v>1.265992745448691</v>
+      </c>
+      <c r="M27" t="n">
+        <v>-0.241655369108422</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>3min</t>
+        </is>
+      </c>
+      <c r="Q27" t="n">
+        <v>6</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>14399</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-1.849196998138443e-05</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.1189310402827884</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-0.472567557799225</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-0.07868358580714307</v>
+      </c>
+      <c r="I28" t="n">
+        <v>-0.0006213906085454357</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.07829521667679164</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.5827090431639853</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.1569788024839347</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0.01495842660680249</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>scaled_first_difference</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>1</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>14398</v>
+      </c>
+      <c r="E29" t="n">
+        <v>-2.027352676513924e-05</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.121858156031165</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-0.5320657085675018</v>
+      </c>
+      <c r="H29" t="n">
+        <v>-0.08015938850243048</v>
+      </c>
+      <c r="I29" t="n">
+        <v>-5.551115123125783e-17</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.08124682206739822</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.5389010052615121</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0.1614062105698287</v>
+      </c>
+      <c r="M29" t="n">
+        <v>-0.02177960641949489</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>scaled_second_difference</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q29" t="n">
+        <v>1</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>subset_B_1min</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>1min</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>7200</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.5531655407698116</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.1661559475541718</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.4530090577120504</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.557426154305987</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.6655566529349839</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1.235552494444517</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0.2125475952229335</v>
+      </c>
+      <c r="M30" t="n">
+        <v>-0.234576655359844</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>scaled_level</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q30" t="n">
+        <v>1</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>1min</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>7199</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.5531662450342165</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.1654217681746355</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.004353419708645234</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.4531942404907017</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.5567828878117247</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.6658457979753343</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1.229574664396824</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0.2126515574846325</v>
+      </c>
+      <c r="M31" t="n">
+        <v>-0.2382941219092898</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>2min</t>
+        </is>
+      </c>
+      <c r="Q31" t="n">
+        <v>2</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>7198</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.5531642817121309</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.1646212245487821</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.004942539191606787</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.4538212628815748</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.5570492911073283</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.6655869752613131</v>
+      </c>
+      <c r="K32" t="n">
+        <v>1.212472872347338</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0.2117657123797383</v>
+      </c>
+      <c r="M32" t="n">
+        <v>-0.2416512443019665</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>3min</t>
+        </is>
+      </c>
+      <c r="Q32" t="n">
+        <v>3</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>7199</v>
+      </c>
+      <c r="E33" t="n">
+        <v>-6.984129575521575e-06</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.03144402132041117</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-0.1289002092240522</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-0.02059752309911399</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.0002469103715357912</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.02070148536081381</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.1428181570090087</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0.04129900845992781</v>
+      </c>
+      <c r="M33" t="n">
+        <v>-0.01495259307717867</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>scaled_first_difference</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q33" t="n">
+        <v>1</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>7198</v>
+      </c>
+      <c r="E34" t="n">
+        <v>-8.003346521805803e-06</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.03601701680820469</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-0.1420124494808386</v>
+      </c>
+      <c r="H34" t="n">
+        <v>-0.02381060674975011</v>
+      </c>
+      <c r="I34" t="n">
+        <v>-0.0002534080128915317</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.02451884965757564</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.1912255851126065</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0.04832945640732574</v>
+      </c>
+      <c r="M34" t="n">
+        <v>-0.006800918693741246</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>scaled_second_difference</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q34" t="n">
+        <v>1</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>minmax</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
         <v>7200</v>
       </c>
-      <c r="E4" t="n">
-        <v>0.9820925256559482</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.9820925256559482</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.8501700577102538</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.7200882547826742</v>
+      <c r="E35" t="n">
+        <v>0.09219850561591178</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.9948555984607741</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-3.219869724328177</v>
+      </c>
+      <c r="H35" t="n">
+        <v>-0.5074865454393293</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.1177088487106715</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.7651381674254907</v>
+      </c>
+      <c r="K35" t="n">
+        <v>4.177977505242388</v>
+      </c>
+      <c r="L35" t="n">
+        <v>1.27262471286482</v>
+      </c>
+      <c r="M35" t="n">
+        <v>-0.2345766553598433</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>scaled_level</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q35" t="n">
+        <v>1</v>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>7199</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.09220272238573905</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.9904597132892966</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-3.19380370602821</v>
+      </c>
+      <c r="H36" t="n">
+        <v>-0.5063777670489563</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.1138573027230665</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.7668694178946689</v>
+      </c>
+      <c r="K36" t="n">
+        <v>4.142185360711084</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1.273247184943625</v>
+      </c>
+      <c r="M36" t="n">
+        <v>-0.2382941219092897</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>2min</t>
+        </is>
+      </c>
+      <c r="Q36" t="n">
+        <v>2</v>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>7198</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.09219096703182313</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.9856664734461507</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-3.190276364248312</v>
+      </c>
+      <c r="H37" t="n">
+        <v>-0.5026234823236587</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.1154523874250022</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.7653197217818091</v>
+      </c>
+      <c r="K37" t="n">
+        <v>4.039788703747625</v>
+      </c>
+      <c r="L37" t="n">
+        <v>1.267943204105468</v>
+      </c>
+      <c r="M37" t="n">
+        <v>-0.241651244301967</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>scaled_trailing_rolling_mean</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>3min</t>
+        </is>
+      </c>
+      <c r="Q37" t="n">
+        <v>3</v>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>7199</v>
+      </c>
+      <c r="E38" t="n">
+        <v>-4.181734395223969e-05</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.1882704838990614</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-0.7717875687086334</v>
+      </c>
+      <c r="H38" t="n">
+        <v>-0.1233272806132794</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.001478371187166427</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.1239497526920893</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.8551210182586974</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0.2472770333053688</v>
+      </c>
+      <c r="M38" t="n">
+        <v>-0.01495259307717845</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>scaled_first_difference</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q38" t="n">
+        <v>1</v>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>7198</v>
+      </c>
+      <c r="E39" t="n">
+        <v>-4.791988617226172e-05</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.2156512080304319</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-0.8502968596479401</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-0.1425655582988612</v>
+      </c>
+      <c r="I39" t="n">
+        <v>-0.001517275692088926</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.1468061493357285</v>
+      </c>
+      <c r="K39" t="n">
+        <v>1.144959579952377</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0.2893717076345896</v>
+      </c>
+      <c r="M39" t="n">
+        <v>-0.006800918693741116</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>TE_8313B.AV_0#</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>scaled_second_difference</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q39" t="n">
+        <v>1</v>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2282,7 +4997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2298,7 +5013,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>transform</t>
+          <t>frequency</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -2308,42 +5023,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>adf_statistic</t>
+          <t>acf_30s</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>adf_pvalue</t>
+          <t>acf_1min</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>adf_used_lag</t>
+          <t>acf_5min</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>adf_nobs</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>kpss_statistic</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>kpss_pvalue</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>kpss_used_lag</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>stationary_recommended</t>
+          <t>acf_10min</t>
         </is>
       </c>
     </row>
@@ -2360,387 +5055,87 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>original</t>
+          <t>5s</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>86400</v>
       </c>
       <c r="E2" t="n">
-        <v>-11.59614553358569</v>
+        <v>0.9916661941774003</v>
       </c>
       <c r="F2" t="n">
-        <v>2.717546204464789e-21</v>
+        <v>0.9773934132442712</v>
       </c>
       <c r="G2" t="n">
-        <v>35</v>
+        <v>0.8456591102333009</v>
       </c>
       <c r="H2" t="n">
-        <v>86364</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.9859335453945668</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K2" t="n">
-        <v>171</v>
-      </c>
-      <c r="L2" t="b">
-        <v>0</v>
+        <v>0.7160959422755356</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>subset_B_raw</t>
+          <t>subset_B_30s</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>30s</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>first_difference</t>
+          <t>30s</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>86399</v>
+        <v>14400</v>
       </c>
       <c r="E3" t="n">
-        <v>-84.37494449290195</v>
+        <v>0.9928528644568304</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>0.9789191558513288</v>
       </c>
       <c r="G3" t="n">
-        <v>5</v>
+        <v>0.8470592565397244</v>
       </c>
       <c r="H3" t="n">
-        <v>86393</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.002386316442035272</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K3" t="n">
-        <v>102</v>
-      </c>
-      <c r="L3" t="b">
-        <v>1</v>
+        <v>0.7173181952148976</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>subset_B_raw</t>
+          <t>subset_B_1min</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>1min</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>second_difference</t>
+          <t>1min</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>86398</v>
+        <v>7200</v>
       </c>
       <c r="E4" t="n">
-        <v>-55.69321961830641</v>
+        <v>0.9820925256559482</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>0.9820925256559482</v>
       </c>
       <c r="G4" t="n">
-        <v>66</v>
+        <v>0.8501700577102538</v>
       </c>
       <c r="H4" t="n">
-        <v>86331</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.01487449827513698</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1751</v>
-      </c>
-      <c r="L4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>subset_B_30s</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>30s</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>original</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>14400</v>
-      </c>
-      <c r="E5" t="n">
-        <v>-8.087124438337199</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1.410039688905484e-12</v>
-      </c>
-      <c r="G5" t="n">
-        <v>25</v>
-      </c>
-      <c r="H5" t="n">
-        <v>14374</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.4536463392403571</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.05403175032743228</v>
-      </c>
-      <c r="K5" t="n">
-        <v>71</v>
-      </c>
-      <c r="L5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>subset_B_30s</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>30s</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>first_difference</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>14399</v>
-      </c>
-      <c r="E6" t="n">
-        <v>-24.35863411902151</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>42</v>
-      </c>
-      <c r="H6" t="n">
-        <v>14356</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.003410636580385386</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K6" t="n">
-        <v>32</v>
-      </c>
-      <c r="L6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>subset_B_30s</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>30s</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>second_difference</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>14398</v>
-      </c>
-      <c r="E7" t="n">
-        <v>-33.05549070761088</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>42</v>
-      </c>
-      <c r="H7" t="n">
-        <v>14355</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.01910025643267669</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K7" t="n">
-        <v>358</v>
-      </c>
-      <c r="L7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>subset_B_1min</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>1min</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>original</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>7200</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-6.738909717850945</v>
-      </c>
-      <c r="F8" t="n">
-        <v>3.155324707751807e-09</v>
-      </c>
-      <c r="G8" t="n">
-        <v>21</v>
-      </c>
-      <c r="H8" t="n">
-        <v>7178</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.3382124415552797</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K8" t="n">
-        <v>51</v>
-      </c>
-      <c r="L8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>subset_B_1min</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>1min</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>first_difference</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>7199</v>
-      </c>
-      <c r="E9" t="n">
-        <v>-23.7558413114052</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>22</v>
-      </c>
-      <c r="H9" t="n">
-        <v>7176</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.004385354410975745</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K9" t="n">
-        <v>23</v>
-      </c>
-      <c r="L9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>subset_B_1min</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>1min</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>second_difference</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>7198</v>
-      </c>
-      <c r="E10" t="n">
-        <v>-26.52043278983831</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>35</v>
-      </c>
-      <c r="H10" t="n">
-        <v>7162</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0.05793038162402646</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K10" t="n">
-        <v>626</v>
-      </c>
-      <c r="L10" t="b">
-        <v>1</v>
+        <v>0.7200882547826742</v>
       </c>
     </row>
   </sheetData>
@@ -2754,6 +5149,478 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id_key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>granularity</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>transform</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>adf_statistic</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>adf_pvalue</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>adf_used_lag</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>adf_nobs</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>kpss_statistic</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>kpss_pvalue</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>kpss_used_lag</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>stationary_recommended</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>86400</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-11.59614553358569</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.717546204464789e-21</v>
+      </c>
+      <c r="G2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H2" t="n">
+        <v>86364</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.9859335453945668</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K2" t="n">
+        <v>171</v>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>first_difference</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>86399</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-84.37494449290195</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>86393</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.002386316442035272</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>102</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>subset_B_raw</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>second_difference</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>86398</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-55.69321961830641</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>66</v>
+      </c>
+      <c r="H4" t="n">
+        <v>86331</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.01487449827513698</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1751</v>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>14400</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-8.087124438337199</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.410039688905484e-12</v>
+      </c>
+      <c r="G5" t="n">
+        <v>25</v>
+      </c>
+      <c r="H5" t="n">
+        <v>14374</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.4536463392403571</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.05403175032743228</v>
+      </c>
+      <c r="K5" t="n">
+        <v>71</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>first_difference</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>14399</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-24.35863411902151</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>42</v>
+      </c>
+      <c r="H6" t="n">
+        <v>14356</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.003410636580385386</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>32</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>subset_B_30s</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>second_difference</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>14398</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-33.05549070761088</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>42</v>
+      </c>
+      <c r="H7" t="n">
+        <v>14355</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.01910025643267669</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>358</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>7200</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-6.738909717850945</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3.155324707751807e-09</v>
+      </c>
+      <c r="G8" t="n">
+        <v>21</v>
+      </c>
+      <c r="H8" t="n">
+        <v>7178</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.3382124415552797</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>51</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>first_difference</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>7199</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-23.7558413114052</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>22</v>
+      </c>
+      <c r="H9" t="n">
+        <v>7176</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.004385354410975745</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>23</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>subset_B_1min</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1min</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>second_difference</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>7198</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-26.52043278983831</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>35</v>
+      </c>
+      <c r="H10" t="n">
+        <v>7162</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.05793038162402646</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>626</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>